<commit_message>
Fix OrgChartTest_ListSchema.xlsx: add the actual Excel Table object
Allan tried importing it and SharePoint's Create List > From Excel
rejected it with "no tables found" — the file had the right data and
formatting but was just styled cells, not a real Excel Table (ListObject).
SharePoint's importer specifically requires a defined Table, which a plain
header-row-plus-cells layout doesn't satisfy no matter how it's styled.

Rebuilt with an actual openpyxl Table ("OrgChartTestData", A1:E11)
wrapping the same 10-post data. Verified the table object round-trips
correctly on read-back before shipping.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/cadets-org-chart/downloads/OrgChartTest_ListSchema.xlsx
+++ b/cadets-org-chart/downloads/OrgChartTest_ListSchema.xlsx
@@ -142,6 +142,20 @@
 </styleSheet>
 </file>
 
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="OrgChartTestData" displayName="OrgChartTestData" ref="A1:E11" headerRowCount="1">
+  <autoFilter ref="A1:E11"/>
+  <tableColumns count="5">
+    <tableColumn id="1" name="Title"/>
+    <tableColumn id="2" name="ManagerPostID"/>
+    <tableColumn id="3" name="SortOrder"/>
+    <tableColumn id="4" name="PostLabel"/>
+    <tableColumn id="5" name="Depth"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -696,5 +710,8 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>